<commit_message>
Added new content from stream, removed extra files.
</commit_message>
<xml_diff>
--- a/Logs/Non Conforming/MDL‑006_NCM_Log.xlsx
+++ b/Logs/Non Conforming/MDL‑006_NCM_Log.xlsx
@@ -78,6 +78,7 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
@@ -99,6 +100,7 @@
       <sz val="14"/>
       <name val="Arial"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -155,23 +157,23 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>

</xml_diff>

<commit_message>
Added new items from stream.
</commit_message>
<xml_diff>
--- a/Logs/Non Conforming/MDL‑006_NCM_Log.xlsx
+++ b/Logs/Non Conforming/MDL‑006_NCM_Log.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="23">
   <si>
     <t xml:space="preserve">Non-Conforming Materials Log</t>
   </si>
@@ -63,6 +63,33 @@
   </si>
   <si>
     <t xml:space="preserve">Disposition By</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MSD</t>
+  </si>
+  <si>
+    <t xml:space="preserve">122925-0001 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">P0001</t>
+  </si>
+  <si>
+    <t xml:space="preserve">JLCPCB</t>
+  </si>
+  <si>
+    <t xml:space="preserve">P1012202501-PCB-01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">N/A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PCB was specified at 2oz copper and was ordered at 1oz copper.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Incoming Inspection</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Use full qty as is</t>
   </si>
 </sst>
 </file>
@@ -413,30 +440,56 @@
       <c r="Y3" s="3"/>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="4"/>
-      <c r="B4" s="2"/>
-      <c r="C4" s="3"/>
+      <c r="A4" s="4" t="n">
+        <v>46020</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>15</v>
+      </c>
       <c r="D4" s="3"/>
-      <c r="E4" s="2"/>
-      <c r="F4" s="2"/>
-      <c r="G4" s="3"/>
+      <c r="E4" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>18</v>
+      </c>
       <c r="H4" s="3"/>
-      <c r="I4" s="3"/>
+      <c r="I4" s="3" t="s">
+        <v>19</v>
+      </c>
       <c r="J4" s="3"/>
-      <c r="K4" s="2"/>
-      <c r="L4" s="3"/>
+      <c r="K4" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="L4" s="3" t="s">
+        <v>20</v>
+      </c>
       <c r="M4" s="3"/>
       <c r="N4" s="3"/>
       <c r="O4" s="3"/>
       <c r="P4" s="3"/>
       <c r="Q4" s="3"/>
-      <c r="R4" s="3"/>
+      <c r="R4" s="3" t="s">
+        <v>21</v>
+      </c>
       <c r="S4" s="3"/>
-      <c r="T4" s="3"/>
+      <c r="T4" s="3" t="s">
+        <v>22</v>
+      </c>
       <c r="U4" s="3"/>
-      <c r="V4" s="5"/>
+      <c r="V4" s="5" t="n">
+        <v>46020</v>
+      </c>
       <c r="W4" s="5"/>
-      <c r="X4" s="3"/>
+      <c r="X4" s="3" t="s">
+        <v>14</v>
+      </c>
       <c r="Y4" s="3"/>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>